<commit_message>
Point marketing 'Source code' links at this deployment's repo; record the production check
The production check after PR #4 found the marketing footer and get-started
page still linking to the upstream repository (BUG-33). AGPL-3.0 section 13
asks for the source users actually run, so they now use SOURCE_URL.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AhDkbZUKfgAGYgJ6gNvp3r
</commit_message>
<xml_diff>
--- a/docs/audit/SM_Bean_QA_Round1_Retest_Engineering.xlsx
+++ b/docs/audit/SM_Bean_QA_Round1_Retest_Engineering.xlsx
@@ -9335,12 +9335,12 @@
       </c>
       <c r="Q2" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: web and worker both on dbe5301 (1 Oct 09:01 UTC)</t>
         </is>
       </c>
       <c r="R2" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -9419,12 +9419,12 @@
       </c>
       <c r="Q3" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Code live; Gmail not connected yet</t>
         </is>
       </c>
       <c r="R3" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4, then connect neopolisinfrallp3@gmail.com at /ops/email/ and send the test email</t>
+          <t>Owner: connect Gmail at /ops/email/, send test email</t>
         </is>
       </c>
     </row>
@@ -9503,12 +9503,12 @@
       </c>
       <c r="Q4" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: pre-deploy backup db-20261001T090041Z.tar.gz in bucket; legacy media 1 copied, 1 lost (vasavi-atlantis-meta-9x16.mp4 404 on old disk)</t>
         </is>
       </c>
       <c r="R4" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4 (release step also copies existing /media files into the bucket)</t>
+          <t>Re-upload that one video</t>
         </is>
       </c>
     </row>
@@ -9587,12 +9587,12 @@
       </c>
       <c r="Q5" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Partly: gunicorn logs now level=info JSON; SENTRY_DSN still unset (W005 at boot)</t>
         </is>
       </c>
       <c r="R5" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4; owner: create Sentry project, set SENTRY_DSN on both services</t>
+          <t>Owner: set SENTRY_DSN</t>
         </is>
       </c>
     </row>
@@ -9671,12 +9671,12 @@
       </c>
       <c r="Q6" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: /accounts/signup/ shows 'invite-only' page</t>
         </is>
       </c>
       <c r="R6" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4; owner: set SIGNUP_ALLOWLIST; delete qa-test-noninvited*@example.com; ACCOUNT_EMAIL_VERIFICATION=mandatory after email works</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -9755,12 +9755,12 @@
       </c>
       <c r="Q7" s="53" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes: worker runs run_worker, 'recurring schedules verified'</t>
         </is>
       </c>
       <c r="R7" s="53" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -9839,12 +9839,12 @@
       </c>
       <c r="Q8" s="53" t="inlineStr">
         <is>
-          <t>Partly</t>
+          <t>Partly: admin reachable from any IP (W010 at boot)</t>
         </is>
       </c>
       <c r="R8" s="53" t="inlineStr">
         <is>
-          <t>Owner: delete DJANGO_SUPERUSER_* vars, rotate admin password, set ADMIN_ALLOWED_IPS</t>
+          <t>Owner: ADMIN_ALLOWED_IPS, delete DJANGO_SUPERUSER_*, rotate password</t>
         </is>
       </c>
     </row>
@@ -9923,12 +9923,12 @@
       </c>
       <c r="Q9" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: /terms/ /privacy/ /support/ 200, own content, no brightbean.xyz</t>
         </is>
       </c>
       <c r="R9" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4; legal review then LEGAL_PAGES_REVIEWED=true</t>
+          <t>Legal review, then LEGAL_PAGES_REVIEWED=true</t>
         </is>
       </c>
     </row>
@@ -10091,12 +10091,12 @@
       </c>
       <c r="Q11" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: GET /accounts/logout/ returns 405</t>
         </is>
       </c>
       <c r="R11" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -10175,7 +10175,7 @@
       </c>
       <c r="Q12" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R12" s="53" t="inlineStr">
@@ -10259,7 +10259,7 @@
       </c>
       <c r="Q13" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R13" s="53" t="inlineStr">
@@ -10343,7 +10343,7 @@
       </c>
       <c r="Q14" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R14" s="53" t="inlineStr">
@@ -10427,7 +10427,7 @@
       </c>
       <c r="Q15" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R15" s="53" t="inlineStr">
@@ -10511,7 +10511,7 @@
       </c>
       <c r="Q16" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R16" s="53" t="inlineStr">
@@ -10595,7 +10595,7 @@
       </c>
       <c r="Q17" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R17" s="53" t="inlineStr">
@@ -10679,7 +10679,7 @@
       </c>
       <c r="Q18" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R18" s="53" t="inlineStr">
@@ -10763,7 +10763,7 @@
       </c>
       <c r="Q19" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R19" s="53" t="inlineStr">
@@ -10847,7 +10847,7 @@
       </c>
       <c r="Q20" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R20" s="53" t="inlineStr">
@@ -10931,7 +10931,7 @@
       </c>
       <c r="Q21" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R21" s="53" t="inlineStr">
@@ -11011,7 +11011,7 @@
       </c>
       <c r="Q22" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R22" s="53" t="inlineStr">
@@ -11095,7 +11095,7 @@
       </c>
       <c r="Q23" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R23" s="53" t="inlineStr">
@@ -11179,12 +11179,12 @@
       </c>
       <c r="Q24" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes on login, signup, marketing; marketing 'Source code' links still went to upstream repo: fixed in PR #5</t>
         </is>
       </c>
       <c r="R24" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4</t>
+          <t>Merge PR #5</t>
         </is>
       </c>
     </row>
@@ -11263,12 +11263,12 @@
       </c>
       <c r="Q25" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: branded 404; invalid portal link shows 'This link isn't valid'</t>
         </is>
       </c>
       <c r="R25" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -11347,12 +11347,12 @@
       </c>
       <c r="Q26" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: robots.txt + sitemap, page titles on every public page</t>
         </is>
       </c>
       <c r="R26" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -11515,7 +11515,7 @@
       </c>
       <c r="Q28" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R28" s="53" t="inlineStr">
@@ -11595,7 +11595,7 @@
       </c>
       <c r="Q29" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R29" s="53" t="inlineStr">
@@ -11675,7 +11675,7 @@
       </c>
       <c r="Q30" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R30" s="53" t="inlineStr">
@@ -11751,7 +11751,7 @@
       </c>
       <c r="Q31" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R31" s="53" t="inlineStr">
@@ -11831,12 +11831,12 @@
       </c>
       <c r="Q32" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: gunicorn booted, /health/ 200 with database+cache checks</t>
         </is>
       </c>
       <c r="R32" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -11911,12 +11911,12 @@
       </c>
       <c r="Q33" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: release ran backup then 8 migrations then media import; worker errors stopped</t>
         </is>
       </c>
       <c r="R33" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4 (worker errors stop once migrate runs)</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -11991,12 +11991,12 @@
       </c>
       <c r="Q34" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes except 'Source code' links → upstream repo; fixed in PR #5</t>
         </is>
       </c>
       <c r="R34" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4; product decision on the self-host page</t>
+          <t>Merge PR #5; product decision on self-host page</t>
         </is>
       </c>
     </row>
@@ -12079,12 +12079,12 @@
       </c>
       <c r="Q35" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: media_library.0004 applied OK on production data</t>
         </is>
       </c>
       <c r="R35" s="53" t="inlineStr">
         <is>
-          <t>Merge PR #4</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -12167,12 +12167,12 @@
       </c>
       <c r="Q36" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: worker live; first cycle 'Generated 0 recurring posts' (no surprise clones)</t>
         </is>
       </c>
       <c r="R36" s="53" t="inlineStr">
         <is>
-          <t>Merge PR #4</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Marketing "Source code" links point at this repo; production check after PR #4 (#5)
The production check after PR #4 found the marketing footer and get-started
page still linking to the upstream repository (BUG-33). AGPL-3.0 section 13
asks for the source users actually run, so they now use SOURCE_URL.


Claude-Session: https://claude.ai/code/session_01AhDkbZUKfgAGYgJ6gNvp3r

Co-authored-by: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/audit/SM_Bean_QA_Round1_Retest_Engineering.xlsx
+++ b/docs/audit/SM_Bean_QA_Round1_Retest_Engineering.xlsx
@@ -9335,12 +9335,12 @@
       </c>
       <c r="Q2" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: web and worker both on dbe5301 (1 Oct 09:01 UTC)</t>
         </is>
       </c>
       <c r="R2" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -9419,12 +9419,12 @@
       </c>
       <c r="Q3" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Code live; Gmail not connected yet</t>
         </is>
       </c>
       <c r="R3" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4, then connect neopolisinfrallp3@gmail.com at /ops/email/ and send the test email</t>
+          <t>Owner: connect Gmail at /ops/email/, send test email</t>
         </is>
       </c>
     </row>
@@ -9503,12 +9503,12 @@
       </c>
       <c r="Q4" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: pre-deploy backup db-20261001T090041Z.tar.gz in bucket; legacy media 1 copied, 1 lost (vasavi-atlantis-meta-9x16.mp4 404 on old disk)</t>
         </is>
       </c>
       <c r="R4" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4 (release step also copies existing /media files into the bucket)</t>
+          <t>Re-upload that one video</t>
         </is>
       </c>
     </row>
@@ -9587,12 +9587,12 @@
       </c>
       <c r="Q5" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Partly: gunicorn logs now level=info JSON; SENTRY_DSN still unset (W005 at boot)</t>
         </is>
       </c>
       <c r="R5" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4; owner: create Sentry project, set SENTRY_DSN on both services</t>
+          <t>Owner: set SENTRY_DSN</t>
         </is>
       </c>
     </row>
@@ -9671,12 +9671,12 @@
       </c>
       <c r="Q6" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: /accounts/signup/ shows 'invite-only' page</t>
         </is>
       </c>
       <c r="R6" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4; owner: set SIGNUP_ALLOWLIST; delete qa-test-noninvited*@example.com; ACCOUNT_EMAIL_VERIFICATION=mandatory after email works</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -9755,12 +9755,12 @@
       </c>
       <c r="Q7" s="53" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>Yes: worker runs run_worker, 'recurring schedules verified'</t>
         </is>
       </c>
       <c r="R7" s="53" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -9839,12 +9839,12 @@
       </c>
       <c r="Q8" s="53" t="inlineStr">
         <is>
-          <t>Partly</t>
+          <t>Partly: admin reachable from any IP (W010 at boot)</t>
         </is>
       </c>
       <c r="R8" s="53" t="inlineStr">
         <is>
-          <t>Owner: delete DJANGO_SUPERUSER_* vars, rotate admin password, set ADMIN_ALLOWED_IPS</t>
+          <t>Owner: ADMIN_ALLOWED_IPS, delete DJANGO_SUPERUSER_*, rotate password</t>
         </is>
       </c>
     </row>
@@ -9923,12 +9923,12 @@
       </c>
       <c r="Q9" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: /terms/ /privacy/ /support/ 200, own content, no brightbean.xyz</t>
         </is>
       </c>
       <c r="R9" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4; legal review then LEGAL_PAGES_REVIEWED=true</t>
+          <t>Legal review, then LEGAL_PAGES_REVIEWED=true</t>
         </is>
       </c>
     </row>
@@ -10091,12 +10091,12 @@
       </c>
       <c r="Q11" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: GET /accounts/logout/ returns 405</t>
         </is>
       </c>
       <c r="R11" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -10175,7 +10175,7 @@
       </c>
       <c r="Q12" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R12" s="53" t="inlineStr">
@@ -10259,7 +10259,7 @@
       </c>
       <c r="Q13" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R13" s="53" t="inlineStr">
@@ -10343,7 +10343,7 @@
       </c>
       <c r="Q14" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R14" s="53" t="inlineStr">
@@ -10427,7 +10427,7 @@
       </c>
       <c r="Q15" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R15" s="53" t="inlineStr">
@@ -10511,7 +10511,7 @@
       </c>
       <c r="Q16" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R16" s="53" t="inlineStr">
@@ -10595,7 +10595,7 @@
       </c>
       <c r="Q17" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R17" s="53" t="inlineStr">
@@ -10679,7 +10679,7 @@
       </c>
       <c r="Q18" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R18" s="53" t="inlineStr">
@@ -10763,7 +10763,7 @@
       </c>
       <c r="Q19" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R19" s="53" t="inlineStr">
@@ -10847,7 +10847,7 @@
       </c>
       <c r="Q20" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R20" s="53" t="inlineStr">
@@ -10931,7 +10931,7 @@
       </c>
       <c r="Q21" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R21" s="53" t="inlineStr">
@@ -11011,7 +11011,7 @@
       </c>
       <c r="Q22" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R22" s="53" t="inlineStr">
@@ -11095,7 +11095,7 @@
       </c>
       <c r="Q23" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R23" s="53" t="inlineStr">
@@ -11179,12 +11179,12 @@
       </c>
       <c r="Q24" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes on login, signup, marketing; marketing 'Source code' links still went to upstream repo: fixed in PR #5</t>
         </is>
       </c>
       <c r="R24" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4</t>
+          <t>Merge PR #5</t>
         </is>
       </c>
     </row>
@@ -11263,12 +11263,12 @@
       </c>
       <c r="Q25" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: branded 404; invalid portal link shows 'This link isn't valid'</t>
         </is>
       </c>
       <c r="R25" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -11347,12 +11347,12 @@
       </c>
       <c r="Q26" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: robots.txt + sitemap, page titles on every public page</t>
         </is>
       </c>
       <c r="R26" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -11515,7 +11515,7 @@
       </c>
       <c r="Q28" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R28" s="53" t="inlineStr">
@@ -11595,7 +11595,7 @@
       </c>
       <c r="Q29" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R29" s="53" t="inlineStr">
@@ -11675,7 +11675,7 @@
       </c>
       <c r="Q30" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R30" s="53" t="inlineStr">
@@ -11751,7 +11751,7 @@
       </c>
       <c r="Q31" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes (dbe5301, 1 Oct). Behind login: needs QA retest signed in</t>
         </is>
       </c>
       <c r="R31" s="53" t="inlineStr">
@@ -11831,12 +11831,12 @@
       </c>
       <c r="Q32" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: gunicorn booted, /health/ 200 with database+cache checks</t>
         </is>
       </c>
       <c r="R32" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -11911,12 +11911,12 @@
       </c>
       <c r="Q33" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: release ran backup then 8 migrations then media import; worker errors stopped</t>
         </is>
       </c>
       <c r="R33" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4 (worker errors stop once migrate runs)</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -11991,12 +11991,12 @@
       </c>
       <c r="Q34" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes except 'Source code' links → upstream repo; fixed in PR #5</t>
         </is>
       </c>
       <c r="R34" s="53" t="inlineStr">
         <is>
-          <t>Deploy PR #4; product decision on the self-host page</t>
+          <t>Merge PR #5; product decision on self-host page</t>
         </is>
       </c>
     </row>
@@ -12079,12 +12079,12 @@
       </c>
       <c r="Q35" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: media_library.0004 applied OK on production data</t>
         </is>
       </c>
       <c r="R35" s="53" t="inlineStr">
         <is>
-          <t>Merge PR #4</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>
@@ -12167,12 +12167,12 @@
       </c>
       <c r="Q36" s="53" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes: worker live; first cycle 'Generated 0 recurring posts' (no surprise clones)</t>
         </is>
       </c>
       <c r="R36" s="53" t="inlineStr">
         <is>
-          <t>Merge PR #4</t>
+          <t>Closed</t>
         </is>
       </c>
     </row>

</xml_diff>